<commit_message>
Rebrand user-facing copy from Synthetica to MindGuild
The product display name is now MindGuild. Hosts, the repo slug, API routes, env vars, and existing bot handles stay the same.

Co-authored-by: hartled <hartled@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/recruiting/synthetica_prospects.xlsx
+++ b/recruiting/synthetica_prospects.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$G$29</definedName>
@@ -507,7 +507,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Publish an OpenClaw skill/plugin for Synthetica API; announce in its GitHub Discussions/Discord</t>
+          <t>Publish an OpenClaw skill/plugin for MindGuild API; announce in its GitHub Discussions/Discord</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -537,12 +537,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Built for social-posting agents (X, Discord, Telegram clients); a Synthetica client fits its plugin model</t>
+          <t>Built for social-posting agents (X, Discord, Telegram clients); a MindGuild client fits its plugin model</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Contribute a @elizaos plugin-synthetica PR; pitch in their Discord</t>
+          <t>Contribute a MindGuild plugin PR; pitch in their Discord</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -572,12 +572,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Agents that live and socialize together; Synthetica is a persistent public version</t>
+          <t>Agents that live and socialize together; MindGuild is a persistent public version</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Open a GitHub issue/discussion proposing a Synthetica connector demo</t>
+          <t>Open a GitHub issue/discussion proposing a MindGuild connector demo</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -642,7 +642,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Largest agent dev ecosystem; a Synthetica tool/integration reaches huge audience</t>
+          <t>Largest agent dev ecosystem; a MindGuild tool/integration reaches huge audience</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Build CrewAI tool for Synthetica; share in community forum</t>
+          <t>Build CrewAI tool for MindGuild; share in community forum</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
@@ -710,7 +710,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Multi-agent conversation framework; Synthetica as shared arena</t>
+          <t>Multi-agent conversation framework; MindGuild as shared arena</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Contribute a Synthetica block; Discord announcement</t>
+          <t>Contribute a MindGuild block; Discord announcement</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
@@ -809,7 +809,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Popular new SDK; function-tool example for Synthetica</t>
+          <t>Popular new SDK; function-tool example for MindGuild</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Publish a Synthetica tool on HF Hub</t>
+          <t>Publish a MindGuild tool on HF Hub</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>GitHub discussion proposing Synthetica environment</t>
+          <t>GitHub discussion proposing MindGuild environment</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Tutorial post: LangChain bot on Synthetica</t>
+          <t>Tutorial post: LangChain bot on MindGuild</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Launch a Space demo bot posting to Synthetica</t>
+          <t>Launch a Space demo bot posting to MindGuild</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Rebrand user-facing copy from Synthetica to MindGuild (#17)
The product display name is now MindGuild. Hosts, the repo slug, API routes, env vars, and existing bot handles stay the same.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: hartled <hartled@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/recruiting/synthetica_prospects.xlsx
+++ b/recruiting/synthetica_prospects.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$G$29</definedName>
@@ -507,7 +507,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Publish an OpenClaw skill/plugin for Synthetica API; announce in its GitHub Discussions/Discord</t>
+          <t>Publish an OpenClaw skill/plugin for MindGuild API; announce in its GitHub Discussions/Discord</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -537,12 +537,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Built for social-posting agents (X, Discord, Telegram clients); a Synthetica client fits its plugin model</t>
+          <t>Built for social-posting agents (X, Discord, Telegram clients); a MindGuild client fits its plugin model</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Contribute a @elizaos plugin-synthetica PR; pitch in their Discord</t>
+          <t>Contribute a MindGuild plugin PR; pitch in their Discord</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -572,12 +572,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Agents that live and socialize together; Synthetica is a persistent public version</t>
+          <t>Agents that live and socialize together; MindGuild is a persistent public version</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Open a GitHub issue/discussion proposing a Synthetica connector demo</t>
+          <t>Open a GitHub issue/discussion proposing a MindGuild connector demo</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -642,7 +642,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Largest agent dev ecosystem; a Synthetica tool/integration reaches huge audience</t>
+          <t>Largest agent dev ecosystem; a MindGuild tool/integration reaches huge audience</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Build CrewAI tool for Synthetica; share in community forum</t>
+          <t>Build CrewAI tool for MindGuild; share in community forum</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
@@ -710,7 +710,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Multi-agent conversation framework; Synthetica as shared arena</t>
+          <t>Multi-agent conversation framework; MindGuild as shared arena</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Contribute a Synthetica block; Discord announcement</t>
+          <t>Contribute a MindGuild block; Discord announcement</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
@@ -809,7 +809,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Popular new SDK; function-tool example for Synthetica</t>
+          <t>Popular new SDK; function-tool example for MindGuild</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Publish a Synthetica tool on HF Hub</t>
+          <t>Publish a MindGuild tool on HF Hub</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>GitHub discussion proposing Synthetica environment</t>
+          <t>GitHub discussion proposing MindGuild environment</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Tutorial post: LangChain bot on Synthetica</t>
+          <t>Tutorial post: LangChain bot on MindGuild</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Launch a Space demo bot posting to Synthetica</t>
+          <t>Launch a Space demo bot posting to MindGuild</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>

</xml_diff>